<commit_message>
Rework Slack auditor to Department + Level model
People sheet now has Department (comma-separated for crossbreeds) and
Level (SWAT, Manager, Lead, Member) columns. Expected channels are the
union of all department channels + level channels. Departments and
Levels each have their own mapping sheet. Template pre-filled with
live channel list for easy assignment.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/references/slack-template.xlsx
+++ b/references/slack-template.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="People" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Roles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Departments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Levels" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +35,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="009AA5B1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -67,10 +74,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,13 +444,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,7 +472,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
         </is>
       </c>
     </row>
@@ -485,7 +499,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Leadership, Sales</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
         </is>
       </c>
     </row>
@@ -507,7 +526,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Rep</t>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Member</t>
         </is>
       </c>
     </row>
@@ -522,17 +546,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Department</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -544,48 +568,478 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>all-aptel</t>
+          <t>-leadership</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>critical-items</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Rep</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>all-aptel</t>
+          <t>development</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Rep</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>22358-elevate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>all-qc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>qc-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>-all-recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>EStream</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>all-estream</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>--- Available Channels ---</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>-all-recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>22358-elevate</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>all-estream</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>all-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>all-qc</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>all-swat</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
           <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>critical-items</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>development</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>qc-managers</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>all-swat</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>all-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>all-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>--- Available Channels ---</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>-all-recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>22358-elevate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>all-estream</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>all-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>all-qc</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>all-swat</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>critical-items</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>development</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>qc-managers</t>
         </is>
       </c>
     </row>

</xml_diff>